<commit_message>
chore: update EU label field to ItemNo
</commit_message>
<xml_diff>
--- a/templates/欧代标签-乘胜-122.xlsx
+++ b/templates/欧代标签-乘胜-122.xlsx
@@ -1597,8 +1597,10 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" s="2" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>ItemNo：</t>
+        </is>
       </c>
       <c r="B2" s="8"/>
     </row>

</xml_diff>